<commit_message>
Updated figures including PPC diagnostic and removed large Rdata from tracking
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Table_S1.xlsx
+++ b/data/Table_S1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://naturalhistorymuseum-my.sharepoint.com/personal/m_stervander_nhm_ac_uk/Documents/Side projects/Great Auk/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ctf150/Dropbox/Research/auk/avi_family_flight_genomics/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="902" documentId="8_{189DF8B4-D90C-4D46-A9EE-1E27D02AC456}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1A777220-03CD-5A44-B7A0-D93C58ED885D}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{985C20C4-4FD9-F042-AC28-E413822EBD66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6040" yWindow="1660" windowWidth="30260" windowHeight="17520" xr2:uid="{C9AD26C9-34CC-B041-B266-8F8DD5E79945}"/>
+    <workbookView xWindow="1260" yWindow="1660" windowWidth="28980" windowHeight="17520" activeTab="1" xr2:uid="{C9AD26C9-34CC-B041-B266-8F8DD5E79945}"/>
   </bookViews>
   <sheets>
     <sheet name="Caption Table S1" sheetId="7" r:id="rId1"/>
@@ -1013,7 +1013,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0000"/>
-    <numFmt numFmtId="166" formatCode="#,##0.0"/>
+    <numFmt numFmtId="165" formatCode="#,##0.0"/>
   </numFmts>
   <fonts count="24" x14ac:knownFonts="1">
     <font>
@@ -1404,7 +1404,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="176">
+  <cellXfs count="163">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1479,19 +1479,19 @@
     <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="166" fontId="5" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" indent="1"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="4" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" indent="1"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" indent="1"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="3" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" indent="1"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1544,35 +1544,17 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" indent="1"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="4" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" indent="1"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1582,79 +1564,37 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" indent="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" indent="1"/>
-    </xf>
     <xf numFmtId="3" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" indent="1"/>
     </xf>
+    <xf numFmtId="3" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
     <xf numFmtId="3" fontId="5" fillId="4" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" indent="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" indent="1"/>
-    </xf>
     <xf numFmtId="3" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" indent="1"/>
     </xf>
+    <xf numFmtId="3" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
     <xf numFmtId="3" fontId="5" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" indent="1"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1668,10 +1608,10 @@
       <alignment horizontal="right" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="5" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" indent="1"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="4" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" indent="1"/>
     </xf>
     <xf numFmtId="3" fontId="5" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1681,10 +1621,10 @@
     <xf numFmtId="164" fontId="5" fillId="3" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" indent="1"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="3" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" indent="1"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="3" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" indent="1"/>
     </xf>
     <xf numFmtId="3" fontId="5" fillId="3" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1692,21 +1632,8 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
@@ -1720,10 +1647,10 @@
     <xf numFmtId="0" fontId="5" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="5" fillId="4" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" indent="1"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="4" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" indent="1"/>
     </xf>
     <xf numFmtId="3" fontId="5" fillId="4" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1735,10 +1662,10 @@
       <alignment horizontal="right" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="5" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" indent="1"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="3" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" indent="1"/>
     </xf>
     <xf numFmtId="3" fontId="5" fillId="3" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1750,8 +1677,6 @@
     <xf numFmtId="0" fontId="5" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1768,6 +1693,60 @@
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -2118,38 +2097,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" ht="165" x14ac:dyDescent="0.2">
-      <c r="A1" s="173" t="s">
+      <c r="A1" s="142" t="s">
         <v>224</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A2" s="174"/>
+      <c r="A2" s="143"/>
     </row>
     <row r="3" spans="1:1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A3" s="174" t="s">
+      <c r="A3" s="143" t="s">
         <v>225</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A4" s="174"/>
+      <c r="A4" s="143"/>
     </row>
     <row r="5" spans="1:1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A5" s="173" t="s">
+      <c r="A5" s="142" t="s">
         <v>226</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="20" x14ac:dyDescent="0.2">
-      <c r="A6" s="175" t="s">
+      <c r="A6" s="144" t="s">
         <v>227</v>
       </c>
     </row>
     <row r="7" spans="1:1" ht="37" x14ac:dyDescent="0.2">
-      <c r="A7" s="175" t="s">
+      <c r="A7" s="144" t="s">
         <v>228</v>
       </c>
     </row>
     <row r="8" spans="1:1" ht="37" x14ac:dyDescent="0.2">
-      <c r="A8" s="175" t="s">
+      <c r="A8" s="144" t="s">
         <v>229</v>
       </c>
     </row>
@@ -2165,7 +2144,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9530F4C2-2FC8-644B-A3AB-0650EA11BB87}">
-  <dimension ref="A1:AZ89"/>
+  <dimension ref="A1:AG89"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7" style="1" customWidth="1"/>
@@ -2195,56 +2174,56 @@
     <col min="29" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" s="91" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="84"/>
-      <c r="B1" s="85"/>
-      <c r="C1" s="85"/>
-      <c r="D1" s="86" t="s">
+    <row r="1" spans="1:28" s="80" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="78"/>
+      <c r="B1" s="147"/>
+      <c r="C1" s="147"/>
+      <c r="D1" s="148" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="87"/>
-      <c r="F1" s="87"/>
-      <c r="G1" s="87"/>
-      <c r="H1" s="87"/>
-      <c r="I1" s="87"/>
-      <c r="J1" s="87"/>
-      <c r="K1" s="87"/>
-      <c r="L1" s="87"/>
-      <c r="M1" s="88"/>
-      <c r="N1" s="88"/>
-      <c r="O1" s="102" t="s">
+      <c r="E1" s="149"/>
+      <c r="F1" s="149"/>
+      <c r="G1" s="149"/>
+      <c r="H1" s="149"/>
+      <c r="I1" s="149"/>
+      <c r="J1" s="149"/>
+      <c r="K1" s="149"/>
+      <c r="L1" s="149"/>
+      <c r="M1" s="79"/>
+      <c r="N1" s="79"/>
+      <c r="O1" s="150" t="s">
         <v>2</v>
       </c>
-      <c r="P1" s="103"/>
-      <c r="Q1" s="103"/>
-      <c r="R1" s="103"/>
-      <c r="S1" s="103"/>
-      <c r="T1" s="103"/>
-      <c r="U1" s="104"/>
-      <c r="V1" s="104"/>
-      <c r="W1" s="104"/>
-      <c r="X1" s="104"/>
-      <c r="Y1" s="105"/>
-      <c r="Z1" s="86" t="s">
+      <c r="P1" s="151"/>
+      <c r="Q1" s="151"/>
+      <c r="R1" s="151"/>
+      <c r="S1" s="151"/>
+      <c r="T1" s="151"/>
+      <c r="U1" s="152"/>
+      <c r="V1" s="152"/>
+      <c r="W1" s="152"/>
+      <c r="X1" s="152"/>
+      <c r="Y1" s="153"/>
+      <c r="Z1" s="148" t="s">
         <v>3</v>
       </c>
-      <c r="AA1" s="89"/>
-      <c r="AB1" s="90"/>
+      <c r="AA1" s="154"/>
+      <c r="AB1" s="155"/>
     </row>
     <row r="2" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="57" t="s">
         <v>199</v>
       </c>
-      <c r="B2" s="78" t="s">
+      <c r="B2" s="156" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="78"/>
+      <c r="C2" s="156"/>
       <c r="D2" s="53"/>
       <c r="E2" s="53"/>
-      <c r="F2" s="70" t="s">
+      <c r="F2" s="157" t="s">
         <v>8</v>
       </c>
-      <c r="G2" s="71"/>
+      <c r="G2" s="158"/>
       <c r="H2" s="51" t="s">
         <v>197</v>
       </c>
@@ -2252,20 +2231,20 @@
       <c r="J2" s="51" t="s">
         <v>194</v>
       </c>
-      <c r="K2" s="73" t="s">
+      <c r="K2" s="159" t="s">
         <v>196</v>
       </c>
-      <c r="L2" s="69"/>
-      <c r="M2" s="73" t="s">
+      <c r="L2" s="160"/>
+      <c r="M2" s="159" t="s">
         <v>214</v>
       </c>
-      <c r="N2" s="69"/>
+      <c r="N2" s="160"/>
       <c r="O2" s="56"/>
       <c r="P2" s="55"/>
-      <c r="Q2" s="72" t="s">
+      <c r="Q2" s="161" t="s">
         <v>8</v>
       </c>
-      <c r="R2" s="71"/>
+      <c r="R2" s="158"/>
       <c r="S2" s="52" t="s">
         <v>197</v>
       </c>
@@ -2273,14 +2252,14 @@
       <c r="U2" s="52" t="s">
         <v>194</v>
       </c>
-      <c r="V2" s="106" t="s">
+      <c r="V2" s="162" t="s">
         <v>196</v>
       </c>
-      <c r="W2" s="69"/>
-      <c r="X2" s="96" t="s">
+      <c r="W2" s="160"/>
+      <c r="X2" s="145" t="s">
         <v>214</v>
       </c>
-      <c r="Y2" s="97"/>
+      <c r="Y2" s="146"/>
       <c r="Z2" s="66"/>
       <c r="AA2" s="67"/>
       <c r="AB2" s="68"/>
@@ -2316,13 +2295,13 @@
       <c r="J3" s="62" t="s">
         <v>201</v>
       </c>
-      <c r="K3" s="74" t="s">
+      <c r="K3" s="69" t="s">
         <v>202</v>
       </c>
       <c r="L3" s="59" t="s">
         <v>203</v>
       </c>
-      <c r="M3" s="74" t="s">
+      <c r="M3" s="69" t="s">
         <v>212</v>
       </c>
       <c r="N3" s="59" t="s">
@@ -2349,13 +2328,13 @@
       <c r="U3" s="63" t="s">
         <v>201</v>
       </c>
-      <c r="V3" s="107" t="s">
+      <c r="V3" s="87" t="s">
         <v>202</v>
       </c>
       <c r="W3" s="60" t="s">
         <v>203</v>
       </c>
-      <c r="X3" s="107" t="s">
+      <c r="X3" s="87" t="s">
         <v>212</v>
       </c>
       <c r="Y3" s="60" t="s">
@@ -2384,7 +2363,7 @@
       <c r="D4" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="79" t="s">
+      <c r="E4" s="73" t="s">
         <v>177</v>
       </c>
       <c r="F4" s="12">
@@ -2398,16 +2377,16 @@
       </c>
       <c r="I4" s="13"/>
       <c r="J4" s="13"/>
-      <c r="K4" s="75">
+      <c r="K4" s="70">
         <v>23900.000002854093</v>
       </c>
       <c r="L4" s="46">
         <v>23450.000000961201</v>
       </c>
-      <c r="M4" s="92">
+      <c r="M4" s="81">
         <v>1164842393.6787701</v>
       </c>
-      <c r="N4" s="92">
+      <c r="N4" s="81">
         <v>15268.134847343201</v>
       </c>
       <c r="O4" s="15" t="s">
@@ -2427,16 +2406,16 @@
       </c>
       <c r="T4" s="10"/>
       <c r="U4" s="10"/>
-      <c r="V4" s="108">
+      <c r="V4" s="88">
         <v>686.18000066462241</v>
       </c>
       <c r="W4" s="48">
         <v>530.86744673834585</v>
       </c>
-      <c r="X4" s="98">
+      <c r="X4" s="84">
         <v>1066908499.57638</v>
       </c>
-      <c r="Y4" s="98">
+      <c r="Y4" s="84">
         <v>15089.589638895501</v>
       </c>
       <c r="Z4" s="17" t="s">
@@ -2472,16 +2451,16 @@
       </c>
       <c r="I5" s="13"/>
       <c r="J5" s="13"/>
-      <c r="K5" s="75">
+      <c r="K5" s="70">
         <v>4399.999995074254</v>
       </c>
       <c r="L5" s="46">
         <v>3369.2133313569648</v>
       </c>
-      <c r="M5" s="92">
+      <c r="M5" s="81">
         <v>1178088651.8929999</v>
       </c>
-      <c r="N5" s="92">
+      <c r="N5" s="81">
         <v>15815.4240793631</v>
       </c>
       <c r="O5" s="15" t="s">
@@ -2505,16 +2484,16 @@
       <c r="U5" s="10" t="s">
         <v>195</v>
       </c>
-      <c r="V5" s="108">
+      <c r="V5" s="88">
         <v>843.41999957955977</v>
       </c>
       <c r="W5" s="48">
         <v>1443.5996853733311</v>
       </c>
-      <c r="X5" s="98">
+      <c r="X5" s="84">
         <v>1257930553.62993</v>
       </c>
-      <c r="Y5" s="98">
+      <c r="Y5" s="84">
         <v>17877.371145958801</v>
       </c>
       <c r="Z5" s="17" t="s">
@@ -2538,7 +2517,7 @@
       <c r="D6" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="E6" s="80" t="s">
+      <c r="E6" s="74" t="s">
         <v>18</v>
       </c>
       <c r="F6" s="12">
@@ -2552,16 +2531,16 @@
       </c>
       <c r="I6" s="13"/>
       <c r="J6" s="13"/>
-      <c r="K6" s="75">
+      <c r="K6" s="70">
         <v>5791.3699987051759</v>
       </c>
       <c r="L6" s="46">
         <v>5658.1849970808089</v>
       </c>
-      <c r="M6" s="92">
+      <c r="M6" s="81">
         <v>1102342267.77581</v>
       </c>
-      <c r="N6" s="92">
+      <c r="N6" s="81">
         <v>14958.5123244925</v>
       </c>
       <c r="O6" s="15" t="s">
@@ -2581,16 +2560,16 @@
       </c>
       <c r="T6" s="10"/>
       <c r="U6" s="10"/>
-      <c r="V6" s="108">
+      <c r="V6" s="88">
         <v>870.08000018550581</v>
       </c>
       <c r="W6" s="48">
         <v>1031.208420763621</v>
       </c>
-      <c r="X6" s="98">
+      <c r="X6" s="84">
         <v>967198391.66388094</v>
       </c>
-      <c r="Y6" s="98">
+      <c r="Y6" s="84">
         <v>15247.831343075901</v>
       </c>
       <c r="Z6" s="17" t="s">
@@ -2616,7 +2595,7 @@
       <c r="D7" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="E7" s="80" t="s">
+      <c r="E7" s="74" t="s">
         <v>18</v>
       </c>
       <c r="F7" s="12">
@@ -2630,16 +2609,16 @@
       </c>
       <c r="I7" s="13"/>
       <c r="J7" s="13"/>
-      <c r="K7" s="75">
+      <c r="K7" s="70">
         <v>751.71999984899333</v>
       </c>
       <c r="L7" s="46">
         <v>438.57347829608267</v>
       </c>
-      <c r="M7" s="92">
+      <c r="M7" s="81">
         <v>1018948750.4742399</v>
       </c>
-      <c r="N7" s="92">
+      <c r="N7" s="81">
         <v>15870.6604852091</v>
       </c>
       <c r="O7" s="15" t="s">
@@ -2661,16 +2640,16 @@
         <v>36</v>
       </c>
       <c r="U7" s="10"/>
-      <c r="V7" s="108">
+      <c r="V7" s="88">
         <v>94.779999920695829</v>
       </c>
       <c r="W7" s="48">
         <v>608.47142851187868</v>
       </c>
-      <c r="X7" s="98">
+      <c r="X7" s="84">
         <v>900903251.90790999</v>
       </c>
-      <c r="Y7" s="98">
+      <c r="Y7" s="84">
         <v>14604.086645802499</v>
       </c>
       <c r="Z7" s="17" t="s">
@@ -2714,16 +2693,16 @@
       <c r="J8" s="13" t="s">
         <v>195</v>
       </c>
-      <c r="K8" s="75">
+      <c r="K8" s="70">
         <v>411.93000012650782</v>
       </c>
       <c r="L8" s="46">
         <v>411.93000012650782</v>
       </c>
-      <c r="M8" s="92">
+      <c r="M8" s="81">
         <v>1197335880.4843199</v>
       </c>
-      <c r="N8" s="92">
+      <c r="N8" s="81">
         <v>15893.765525811301</v>
       </c>
       <c r="O8" s="15" t="s">
@@ -2747,16 +2726,16 @@
       <c r="U8" s="10" t="s">
         <v>195</v>
       </c>
-      <c r="V8" s="108">
+      <c r="V8" s="88">
         <v>730.96000016206062</v>
       </c>
       <c r="W8" s="48">
         <v>555.74166681365045</v>
       </c>
-      <c r="X8" s="98">
+      <c r="X8" s="84">
         <v>1171360458.52423</v>
       </c>
-      <c r="Y8" s="98">
+      <c r="Y8" s="84">
         <v>14646.7522620322</v>
       </c>
       <c r="Z8" s="17" t="s">
@@ -2796,16 +2775,16 @@
       </c>
       <c r="I9" s="13"/>
       <c r="J9" s="13"/>
-      <c r="K9" s="75">
+      <c r="K9" s="70">
         <v>261.23999994663291</v>
       </c>
       <c r="L9" s="46">
         <v>263.22176469505297</v>
       </c>
-      <c r="M9" s="92">
+      <c r="M9" s="81">
         <v>1190974462.6277201</v>
       </c>
-      <c r="N9" s="92">
+      <c r="N9" s="81">
         <v>15242.1040201672</v>
       </c>
       <c r="O9" s="15" t="s">
@@ -2825,16 +2804,16 @@
       </c>
       <c r="T9" s="10"/>
       <c r="U9" s="10"/>
-      <c r="V9" s="108">
+      <c r="V9" s="88">
         <v>964.99000031213927</v>
       </c>
       <c r="W9" s="48">
         <v>431.02500006134505</v>
       </c>
-      <c r="X9" s="98">
+      <c r="X9" s="84">
         <v>1184047588.3066499</v>
       </c>
-      <c r="Y9" s="98">
+      <c r="Y9" s="84">
         <v>15737.4512358353</v>
       </c>
       <c r="Z9" s="17" t="s">
@@ -2874,16 +2853,16 @@
       </c>
       <c r="I10" s="13"/>
       <c r="J10" s="13"/>
-      <c r="K10" s="75">
+      <c r="K10" s="70">
         <v>712.10000037745499</v>
       </c>
       <c r="L10" s="46">
         <v>977.20333327166134</v>
       </c>
-      <c r="M10" s="92">
+      <c r="M10" s="81">
         <v>1111532059.57686</v>
       </c>
-      <c r="N10" s="92">
+      <c r="N10" s="81">
         <v>15523.295099494901</v>
       </c>
       <c r="O10" s="15" t="s">
@@ -2905,16 +2884,16 @@
         <v>26</v>
       </c>
       <c r="U10" s="10"/>
-      <c r="V10" s="108">
+      <c r="V10" s="88">
         <v>1501.3300004120258</v>
       </c>
       <c r="W10" s="48">
         <v>4130.6249976256295</v>
       </c>
-      <c r="X10" s="98">
+      <c r="X10" s="84">
         <v>1112078069.5850301</v>
       </c>
-      <c r="Y10" s="98">
+      <c r="Y10" s="84">
         <v>14761.8464962899</v>
       </c>
       <c r="Z10" s="17" t="s">
@@ -2928,82 +2907,82 @@
       </c>
     </row>
     <row r="11" spans="1:28" s="18" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="110">
+      <c r="A11" s="90">
         <v>8</v>
       </c>
-      <c r="B11" s="111" t="s">
+      <c r="B11" s="91" t="s">
         <v>13</v>
       </c>
-      <c r="C11" s="112" t="s">
+      <c r="C11" s="92" t="s">
         <v>14</v>
       </c>
-      <c r="D11" s="113" t="s">
+      <c r="D11" s="93" t="s">
         <v>50</v>
       </c>
-      <c r="E11" s="114" t="s">
+      <c r="E11" s="94" t="s">
         <v>18</v>
       </c>
-      <c r="F11" s="115">
+      <c r="F11" s="95">
         <v>6.475186807</v>
       </c>
-      <c r="G11" s="115">
+      <c r="G11" s="95">
         <v>23.221053297499999</v>
       </c>
-      <c r="H11" s="116" t="s">
+      <c r="H11" s="96" t="s">
         <v>16</v>
       </c>
-      <c r="I11" s="116"/>
-      <c r="J11" s="116"/>
-      <c r="K11" s="117">
+      <c r="I11" s="96"/>
+      <c r="J11" s="96"/>
+      <c r="K11" s="97">
         <v>376.000000062629</v>
       </c>
-      <c r="L11" s="118">
+      <c r="L11" s="98">
         <v>237.86636364842596</v>
       </c>
-      <c r="M11" s="119">
+      <c r="M11" s="99">
         <v>1234179044.8703799</v>
       </c>
-      <c r="N11" s="119">
+      <c r="N11" s="99">
         <v>15991.547029368099</v>
       </c>
-      <c r="O11" s="120" t="s">
+      <c r="O11" s="100" t="s">
         <v>51</v>
       </c>
-      <c r="P11" s="112" t="s">
-        <v>23</v>
-      </c>
-      <c r="Q11" s="121">
+      <c r="P11" s="92" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q11" s="101">
         <v>19.318631419999999</v>
       </c>
-      <c r="R11" s="121">
+      <c r="R11" s="101">
         <v>10.928604820454545</v>
       </c>
-      <c r="S11" s="112" t="s">
+      <c r="S11" s="92" t="s">
         <v>16</v>
       </c>
-      <c r="T11" s="112" t="s">
+      <c r="T11" s="92" t="s">
         <v>52</v>
       </c>
-      <c r="U11" s="112"/>
-      <c r="V11" s="122">
+      <c r="U11" s="92"/>
+      <c r="V11" s="102">
         <v>82.040000057364779</v>
       </c>
-      <c r="W11" s="123">
+      <c r="W11" s="103">
         <v>120.3450000567523</v>
       </c>
-      <c r="X11" s="124">
+      <c r="X11" s="104">
         <v>1072941785.17237</v>
       </c>
-      <c r="Y11" s="124">
+      <c r="Y11" s="104">
         <v>15079.664261615</v>
       </c>
-      <c r="Z11" s="125" t="s">
+      <c r="Z11" s="105" t="s">
         <v>184</v>
       </c>
-      <c r="AA11" s="116" t="s">
+      <c r="AA11" s="96" t="s">
         <v>53</v>
       </c>
-      <c r="AB11" s="126" t="s">
+      <c r="AB11" s="106" t="s">
         <v>54</v>
       </c>
     </row>
@@ -3011,10 +2990,10 @@
       <c r="A12" s="8" t="s">
         <v>217</v>
       </c>
-      <c r="B12" s="127" t="s">
+      <c r="B12" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="C12" s="127" t="s">
+      <c r="C12" s="19" t="s">
         <v>21</v>
       </c>
       <c r="D12" s="11" t="s">
@@ -3023,64 +3002,64 @@
       <c r="E12" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="F12" s="128">
+      <c r="F12" s="12">
         <v>13.402205110000001</v>
       </c>
-      <c r="G12" s="128">
+      <c r="G12" s="12">
         <v>19.369522499428573</v>
       </c>
-      <c r="H12" s="129" t="s">
+      <c r="H12" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="I12" s="129"/>
-      <c r="J12" s="129"/>
-      <c r="K12" s="75">
+      <c r="I12" s="13"/>
+      <c r="J12" s="13"/>
+      <c r="K12" s="70">
         <v>65.800000058489644</v>
       </c>
       <c r="L12" s="46">
         <v>94.299428562035501</v>
       </c>
-      <c r="M12" s="92">
+      <c r="M12" s="81">
         <v>1129445982.87411</v>
       </c>
-      <c r="N12" s="92">
+      <c r="N12" s="81">
         <v>14258.728059041399</v>
       </c>
       <c r="O12" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="P12" s="130" t="s">
-        <v>23</v>
-      </c>
-      <c r="Q12" s="131">
+      <c r="P12" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q12" s="16">
         <v>49.201626640000001</v>
       </c>
-      <c r="R12" s="131">
+      <c r="R12" s="16">
         <v>36.479997328103451</v>
       </c>
-      <c r="S12" s="127" t="s">
+      <c r="S12" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="T12" s="132" t="s">
+      <c r="T12" s="107" t="s">
         <v>57</v>
       </c>
-      <c r="U12" s="130"/>
-      <c r="V12" s="108">
+      <c r="U12" s="10"/>
+      <c r="V12" s="88">
         <v>111.35999993166865</v>
       </c>
       <c r="W12" s="48">
         <v>75.886153851766878</v>
       </c>
-      <c r="X12" s="98">
+      <c r="X12" s="84">
         <v>1150976505.9448299</v>
       </c>
-      <c r="Y12" s="98">
+      <c r="Y12" s="84">
         <v>14981.042495559501</v>
       </c>
       <c r="Z12" s="17" t="s">
         <v>184</v>
       </c>
-      <c r="AA12" s="129" t="s">
+      <c r="AA12" s="13" t="s">
         <v>53</v>
       </c>
       <c r="AB12" s="14" t="s">
@@ -3091,86 +3070,86 @@
       <c r="A13" s="8">
         <v>10</v>
       </c>
-      <c r="B13" s="133" t="s">
+      <c r="B13" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="C13" s="127" t="s">
+      <c r="C13" s="19" t="s">
         <v>21</v>
       </c>
       <c r="D13" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="E13" s="81" t="s">
+      <c r="E13" s="75" t="s">
         <v>176</v>
       </c>
-      <c r="F13" s="128">
+      <c r="F13" s="12">
         <v>9.1076696170000009</v>
       </c>
-      <c r="G13" s="128">
+      <c r="G13" s="12">
         <v>9.9822511089999999</v>
       </c>
-      <c r="H13" s="129" t="s">
+      <c r="H13" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="I13" s="129"/>
-      <c r="J13" s="129"/>
-      <c r="K13" s="75">
+      <c r="I13" s="13"/>
+      <c r="J13" s="13"/>
+      <c r="K13" s="70">
         <v>147.9999998654055</v>
       </c>
       <c r="L13" s="46">
         <v>132.97999994995396</v>
       </c>
-      <c r="M13" s="92">
+      <c r="M13" s="81">
         <v>1117618984.0558</v>
       </c>
-      <c r="N13" s="92">
+      <c r="N13" s="81">
         <v>15693.788006369299</v>
       </c>
       <c r="O13" s="15" t="s">
         <v>59</v>
       </c>
-      <c r="P13" s="130" t="s">
-        <v>23</v>
-      </c>
-      <c r="Q13" s="131">
+      <c r="P13" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q13" s="16">
         <v>54.206644400000002</v>
       </c>
-      <c r="R13" s="131">
+      <c r="R13" s="16">
         <v>54.434054588750001</v>
       </c>
-      <c r="S13" s="127" t="s">
+      <c r="S13" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="T13" s="134" t="s">
+      <c r="T13" s="45" t="s">
         <v>60</v>
       </c>
-      <c r="U13" s="130"/>
-      <c r="V13" s="108">
+      <c r="U13" s="10"/>
+      <c r="V13" s="88">
         <v>337.99999978390878</v>
       </c>
       <c r="W13" s="48">
         <v>248.22625000977195</v>
       </c>
-      <c r="X13" s="98">
+      <c r="X13" s="84">
         <v>1095795780.9753101</v>
       </c>
-      <c r="Y13" s="98">
+      <c r="Y13" s="84">
         <v>14979.455925365201</v>
       </c>
       <c r="Z13" s="17" t="s">
         <v>185</v>
       </c>
-      <c r="AA13" s="129"/>
+      <c r="AA13" s="13"/>
       <c r="AB13" s="14"/>
     </row>
     <row r="14" spans="1:28" s="18" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A14" s="8">
         <v>11</v>
       </c>
-      <c r="B14" s="127" t="s">
+      <c r="B14" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="C14" s="127" t="s">
+      <c r="C14" s="19" t="s">
         <v>21</v>
       </c>
       <c r="D14" s="11" t="s">
@@ -3179,64 +3158,64 @@
       <c r="E14" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="F14" s="128">
+      <c r="F14" s="12">
         <v>44.180791370000001</v>
       </c>
-      <c r="G14" s="128">
+      <c r="G14" s="12">
         <v>37.017598020800008</v>
       </c>
-      <c r="H14" s="129" t="s">
+      <c r="H14" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="I14" s="129"/>
-      <c r="J14" s="129"/>
-      <c r="K14" s="75">
+      <c r="I14" s="13"/>
+      <c r="J14" s="13"/>
+      <c r="K14" s="70">
         <v>354.20000011902846</v>
       </c>
       <c r="L14" s="46">
         <v>272.0843999604694</v>
       </c>
-      <c r="M14" s="92">
+      <c r="M14" s="81">
         <v>1103041213.5639801</v>
       </c>
-      <c r="N14" s="92">
+      <c r="N14" s="81">
         <v>15051.836823059</v>
       </c>
       <c r="O14" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="P14" s="130" t="s">
-        <v>23</v>
-      </c>
-      <c r="Q14" s="131">
+      <c r="P14" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q14" s="16">
         <v>36.234793099999997</v>
       </c>
-      <c r="R14" s="131">
+      <c r="R14" s="16">
         <v>35.804541989999997</v>
       </c>
-      <c r="S14" s="127" t="s">
+      <c r="S14" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="T14" s="134" t="s">
+      <c r="T14" s="45" t="s">
         <v>60</v>
       </c>
-      <c r="U14" s="130"/>
-      <c r="V14" s="108">
+      <c r="U14" s="10"/>
+      <c r="V14" s="88">
         <v>366.30000028293529</v>
       </c>
       <c r="W14" s="48">
         <v>263.54647055334738</v>
       </c>
-      <c r="X14" s="98">
+      <c r="X14" s="84">
         <v>1069600346.19291</v>
       </c>
-      <c r="Y14" s="98">
+      <c r="Y14" s="84">
         <v>14529.21351955</v>
       </c>
       <c r="Z14" s="17" t="s">
         <v>185</v>
       </c>
-      <c r="AA14" s="129" t="s">
+      <c r="AA14" s="13" t="s">
         <v>63</v>
       </c>
       <c r="AB14" s="14" t="s">
@@ -3247,74 +3226,74 @@
       <c r="A15" s="8">
         <v>12</v>
       </c>
-      <c r="B15" s="133" t="s">
+      <c r="B15" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="C15" s="130" t="s">
+      <c r="C15" s="10" t="s">
         <v>14</v>
       </c>
       <c r="D15" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="E15" s="80" t="s">
+      <c r="E15" s="74" t="s">
         <v>18</v>
       </c>
-      <c r="F15" s="128">
+      <c r="F15" s="12">
         <v>9.6244142789999998</v>
       </c>
-      <c r="G15" s="128">
+      <c r="G15" s="12">
         <v>8.1345912139999985</v>
       </c>
-      <c r="H15" s="129" t="s">
+      <c r="H15" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="I15" s="129"/>
-      <c r="J15" s="129"/>
-      <c r="K15" s="75">
+      <c r="I15" s="13"/>
+      <c r="J15" s="13"/>
+      <c r="K15" s="70">
         <v>1026.0000005296681</v>
       </c>
       <c r="L15" s="46">
         <v>1137.5266674524003</v>
       </c>
-      <c r="M15" s="92">
+      <c r="M15" s="81">
         <v>1174938589.4771399</v>
       </c>
-      <c r="N15" s="92">
+      <c r="N15" s="81">
         <v>15769.094351969399</v>
       </c>
       <c r="O15" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="P15" s="130" t="s">
-        <v>23</v>
-      </c>
-      <c r="Q15" s="131">
+      <c r="P15" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q15" s="16">
         <v>37.97820359</v>
       </c>
-      <c r="R15" s="131">
+      <c r="R15" s="16">
         <v>39.261993049375</v>
       </c>
-      <c r="S15" s="130" t="s">
+      <c r="S15" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="T15" s="135"/>
-      <c r="U15" s="130"/>
-      <c r="V15" s="108">
+      <c r="T15" s="108"/>
+      <c r="U15" s="10"/>
+      <c r="V15" s="88">
         <v>3771.9900026072137</v>
       </c>
       <c r="W15" s="48">
         <v>5025.759376840283</v>
       </c>
-      <c r="X15" s="98">
+      <c r="X15" s="84">
         <v>1154809394.9895501</v>
       </c>
-      <c r="Y15" s="98">
+      <c r="Y15" s="84">
         <v>15239.8769227417</v>
       </c>
       <c r="Z15" s="17" t="s">
         <v>186</v>
       </c>
-      <c r="AA15" s="129" t="s">
+      <c r="AA15" s="13" t="s">
         <v>67</v>
       </c>
       <c r="AB15" s="14"/>
@@ -3323,159 +3302,159 @@
       <c r="A16" s="8" t="s">
         <v>218</v>
       </c>
-      <c r="B16" s="133" t="s">
+      <c r="B16" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="C16" s="130" t="s">
+      <c r="C16" s="10" t="s">
         <v>14</v>
       </c>
       <c r="D16" s="11" t="s">
         <v>179</v>
       </c>
-      <c r="E16" s="79" t="s">
+      <c r="E16" s="73" t="s">
         <v>177</v>
       </c>
-      <c r="F16" s="128">
+      <c r="F16" s="12">
         <v>0.18463009899999999</v>
       </c>
-      <c r="G16" s="128">
+      <c r="G16" s="12">
         <v>22.158963342228347</v>
       </c>
-      <c r="H16" s="136" t="s">
+      <c r="H16" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="I16" s="136"/>
-      <c r="J16" s="129"/>
-      <c r="K16" s="76">
-        <v>39.26999997554811</v>
+      <c r="I16" s="22"/>
+      <c r="J16" s="13"/>
+      <c r="K16" s="71">
+        <v>3560</v>
       </c>
       <c r="L16" s="47">
-        <v>315.01868849786854</v>
-      </c>
-      <c r="M16" s="93">
+        <v>3560</v>
+      </c>
+      <c r="M16" s="82">
         <v>1220854836.1730599</v>
       </c>
-      <c r="N16" s="93">
+      <c r="N16" s="82">
         <v>16353.785226848</v>
       </c>
       <c r="O16" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="P16" s="137" t="s">
-        <v>23</v>
-      </c>
-      <c r="Q16" s="131">
+      <c r="P16" s="24" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q16" s="16">
         <v>36.247463029999999</v>
       </c>
-      <c r="R16" s="131">
+      <c r="R16" s="16">
         <v>21.525801973333333</v>
       </c>
-      <c r="S16" s="137" t="s">
+      <c r="S16" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="T16" s="137"/>
-      <c r="U16" s="130" t="s">
+      <c r="T16" s="24"/>
+      <c r="U16" s="10" t="s">
         <v>195</v>
       </c>
-      <c r="V16" s="108">
+      <c r="V16" s="88">
         <v>131.99999993743378</v>
       </c>
       <c r="W16" s="48">
         <v>129.05166660850594</v>
       </c>
-      <c r="X16" s="99">
+      <c r="X16" s="85">
         <v>1108060246.9022</v>
       </c>
-      <c r="Y16" s="99">
+      <c r="Y16" s="85">
         <v>15506.160908038</v>
       </c>
       <c r="Z16" s="17" t="s">
         <v>186</v>
       </c>
-      <c r="AA16" s="129" t="s">
+      <c r="AA16" s="13" t="s">
         <v>67</v>
       </c>
       <c r="AB16" s="14"/>
     </row>
     <row r="17" spans="1:28" s="18" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="138">
+      <c r="A17" s="109">
         <v>14</v>
       </c>
-      <c r="B17" s="139" t="s">
+      <c r="B17" s="110" t="s">
         <v>37</v>
       </c>
-      <c r="C17" s="140" t="s">
+      <c r="C17" s="111" t="s">
         <v>38</v>
       </c>
-      <c r="D17" s="141" t="s">
+      <c r="D17" s="112" t="s">
         <v>69</v>
       </c>
-      <c r="E17" s="142" t="s">
-        <v>23</v>
-      </c>
-      <c r="F17" s="143">
+      <c r="E17" s="113" t="s">
+        <v>23</v>
+      </c>
+      <c r="F17" s="114">
         <v>52.619160190000002</v>
       </c>
-      <c r="G17" s="143">
+      <c r="G17" s="114">
         <v>52.523437236363634</v>
       </c>
-      <c r="H17" s="144" t="s">
+      <c r="H17" s="115" t="s">
         <v>25</v>
       </c>
-      <c r="I17" s="145" t="s">
+      <c r="I17" s="116" t="s">
         <v>40</v>
       </c>
-      <c r="J17" s="146"/>
-      <c r="K17" s="147">
+      <c r="J17" s="117"/>
+      <c r="K17" s="118">
         <v>96.440000065415703</v>
       </c>
-      <c r="L17" s="148">
+      <c r="L17" s="119">
         <v>64.624545473384259</v>
       </c>
-      <c r="M17" s="149">
+      <c r="M17" s="120">
         <v>1215932822.8123901</v>
       </c>
-      <c r="N17" s="149">
+      <c r="N17" s="120">
         <v>14598.5777923478</v>
       </c>
-      <c r="O17" s="150" t="s">
+      <c r="O17" s="121" t="s">
         <v>180</v>
       </c>
-      <c r="P17" s="151" t="s">
-        <v>23</v>
-      </c>
-      <c r="Q17" s="152">
+      <c r="P17" s="122" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q17" s="123">
         <v>54.985272709999997</v>
       </c>
-      <c r="R17" s="152">
+      <c r="R17" s="123">
         <v>51.981876338695649</v>
       </c>
-      <c r="S17" s="144" t="s">
+      <c r="S17" s="115" t="s">
         <v>25</v>
       </c>
-      <c r="T17" s="153" t="s">
+      <c r="T17" s="124" t="s">
         <v>70</v>
       </c>
-      <c r="U17" s="140"/>
-      <c r="V17" s="154">
+      <c r="U17" s="111"/>
+      <c r="V17" s="125">
         <v>42.299999963471144</v>
       </c>
-      <c r="W17" s="155">
+      <c r="W17" s="126">
         <v>60.025909089823386</v>
       </c>
-      <c r="X17" s="156">
+      <c r="X17" s="127">
         <v>1236848961.0297301</v>
       </c>
-      <c r="Y17" s="156">
+      <c r="Y17" s="127">
         <v>16007.1544764501</v>
       </c>
-      <c r="Z17" s="157" t="s">
+      <c r="Z17" s="128" t="s">
         <v>186</v>
       </c>
-      <c r="AA17" s="146" t="s">
+      <c r="AA17" s="117" t="s">
         <v>71</v>
       </c>
-      <c r="AB17" s="158" t="s">
+      <c r="AB17" s="129" t="s">
         <v>72</v>
       </c>
     </row>
@@ -3492,7 +3471,7 @@
       <c r="D18" s="11" t="s">
         <v>210</v>
       </c>
-      <c r="E18" s="79" t="s">
+      <c r="E18" s="73" t="s">
         <v>177</v>
       </c>
       <c r="F18" s="12">
@@ -3508,16 +3487,16 @@
       <c r="J18" s="13" t="s">
         <v>195</v>
       </c>
-      <c r="K18" s="75">
-        <v>4750</v>
+      <c r="K18" s="70">
+        <v>3560</v>
       </c>
       <c r="L18" s="46">
-        <v>4750</v>
-      </c>
-      <c r="M18" s="94">
+        <v>3560</v>
+      </c>
+      <c r="M18" s="81">
         <v>26111648.131550301</v>
       </c>
-      <c r="N18" s="94">
+      <c r="N18" s="81">
         <v>15646.594324923401</v>
       </c>
       <c r="O18" s="23" t="s">
@@ -3541,16 +3520,16 @@
       <c r="U18" s="10" t="s">
         <v>195</v>
       </c>
-      <c r="V18" s="108">
+      <c r="V18" s="88">
         <v>725.99000059972718</v>
       </c>
       <c r="W18" s="48">
         <v>725.99000059972718</v>
       </c>
-      <c r="X18" s="100">
+      <c r="X18" s="84">
         <v>1175339792.1315501</v>
       </c>
-      <c r="Y18" s="100">
+      <c r="Y18" s="84">
         <v>16095.594324923401</v>
       </c>
       <c r="Z18" s="17" t="s">
@@ -3576,7 +3555,7 @@
       <c r="D19" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="E19" s="81" t="s">
+      <c r="E19" s="75" t="s">
         <v>176</v>
       </c>
       <c r="F19" s="12">
@@ -3590,16 +3569,16 @@
       </c>
       <c r="I19" s="13"/>
       <c r="J19" s="13"/>
-      <c r="K19" s="75">
+      <c r="K19" s="70">
         <v>859.98999944876982</v>
       </c>
       <c r="L19" s="46">
         <v>534.99499978871575</v>
       </c>
-      <c r="M19" s="92">
+      <c r="M19" s="81">
         <v>1117650131.0004699</v>
       </c>
-      <c r="N19" s="92">
+      <c r="N19" s="81">
         <v>15224.6011116681</v>
       </c>
       <c r="O19" s="15" t="s">
@@ -3621,16 +3600,16 @@
         <v>79</v>
       </c>
       <c r="U19" s="10"/>
-      <c r="V19" s="108">
+      <c r="V19" s="88">
         <v>328.03999983065182</v>
       </c>
       <c r="W19" s="48">
         <v>583.30000027521669</v>
       </c>
-      <c r="X19" s="98">
+      <c r="X19" s="84">
         <v>1183155367.63938</v>
       </c>
-      <c r="Y19" s="98">
+      <c r="Y19" s="84">
         <v>15268.4300809134</v>
       </c>
       <c r="Z19" s="17" t="s">
@@ -3652,7 +3631,7 @@
       <c r="D20" s="11" t="s">
         <v>80</v>
       </c>
-      <c r="E20" s="79" t="s">
+      <c r="E20" s="73" t="s">
         <v>177</v>
       </c>
       <c r="F20" s="12">
@@ -3668,16 +3647,16 @@
       <c r="J20" s="13" t="s">
         <v>195</v>
       </c>
-      <c r="K20" s="75">
+      <c r="K20" s="70">
         <v>33569.329970345309</v>
       </c>
       <c r="L20" s="46">
         <v>5911.1049980285643</v>
       </c>
-      <c r="M20" s="92">
+      <c r="M20" s="81">
         <v>1246104098.11099</v>
       </c>
-      <c r="N20" s="92">
+      <c r="N20" s="81">
         <v>14559.664790336101</v>
       </c>
       <c r="O20" s="15" t="s">
@@ -3701,16 +3680,16 @@
       <c r="U20" s="10" t="s">
         <v>195</v>
       </c>
-      <c r="V20" s="108">
+      <c r="V20" s="88">
         <v>152.05999994722319</v>
       </c>
       <c r="W20" s="48">
         <v>1036.625468597744</v>
       </c>
-      <c r="X20" s="98">
+      <c r="X20" s="84">
         <v>1228911136.8915601</v>
       </c>
-      <c r="Y20" s="98">
+      <c r="Y20" s="84">
         <v>16931.649180421198</v>
       </c>
       <c r="Z20" s="17" t="s">
@@ -3732,7 +3711,7 @@
       <c r="D21" s="11" t="s">
         <v>181</v>
       </c>
-      <c r="E21" s="79" t="s">
+      <c r="E21" s="73" t="s">
         <v>177</v>
       </c>
       <c r="F21" s="12">
@@ -3748,16 +3727,16 @@
       <c r="J21" s="13" t="s">
         <v>195</v>
       </c>
-      <c r="K21" s="76">
+      <c r="K21" s="71">
         <v>3016.6199995422653</v>
       </c>
       <c r="L21" s="47">
         <v>2050.4300004835709</v>
       </c>
-      <c r="M21" s="93">
+      <c r="M21" s="82">
         <v>1192134113.12672</v>
       </c>
-      <c r="N21" s="93">
+      <c r="N21" s="82">
         <v>16170.983685412901</v>
       </c>
       <c r="O21" s="23" t="s">
@@ -3781,16 +3760,16 @@
       <c r="U21" s="10" t="s">
         <v>195</v>
       </c>
-      <c r="V21" s="108">
+      <c r="V21" s="88">
         <v>2528.9700026749633</v>
       </c>
       <c r="W21" s="48">
         <v>1701.7278577689453</v>
       </c>
-      <c r="X21" s="99">
+      <c r="X21" s="85">
         <v>1171072281.4948001</v>
       </c>
-      <c r="Y21" s="99">
+      <c r="Y21" s="85">
         <v>14442.322374466699</v>
       </c>
       <c r="Z21" s="17" t="s">
@@ -3830,16 +3809,16 @@
       </c>
       <c r="I22" s="13"/>
       <c r="J22" s="13"/>
-      <c r="K22" s="75">
+      <c r="K22" s="70">
         <v>756.00000086827697</v>
       </c>
       <c r="L22" s="46">
         <v>1179.3425000782379</v>
       </c>
-      <c r="M22" s="92">
+      <c r="M22" s="81">
         <v>1206704702.2111299</v>
       </c>
-      <c r="N22" s="92">
+      <c r="N22" s="81">
         <v>16103.066567985001</v>
       </c>
       <c r="O22" s="15" t="s">
@@ -3861,16 +3840,16 @@
         <v>89</v>
       </c>
       <c r="U22" s="10"/>
-      <c r="V22" s="108">
+      <c r="V22" s="88">
         <v>1900.0000002063712</v>
       </c>
       <c r="W22" s="48">
         <v>1396.2252001106829</v>
       </c>
-      <c r="X22" s="98">
+      <c r="X22" s="84">
         <v>1245255772.0404699</v>
       </c>
-      <c r="Y22" s="98">
+      <c r="Y22" s="84">
         <v>14519.970453236199</v>
       </c>
       <c r="Z22" s="17" t="s">
@@ -3896,7 +3875,7 @@
       <c r="D23" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="E23" s="82" t="s">
+      <c r="E23" s="76" t="s">
         <v>23</v>
       </c>
       <c r="F23" s="12">
@@ -3910,16 +3889,16 @@
       </c>
       <c r="I23" s="22"/>
       <c r="J23" s="13"/>
-      <c r="K23" s="75">
+      <c r="K23" s="70">
         <v>472.00000039768133</v>
       </c>
       <c r="L23" s="46">
         <v>472.00000039768133</v>
       </c>
-      <c r="M23" s="92">
+      <c r="M23" s="81">
         <v>1150644276.7462399</v>
       </c>
-      <c r="N23" s="92">
+      <c r="N23" s="81">
         <v>15051.435374283999</v>
       </c>
       <c r="O23" s="23" t="s">
@@ -3943,16 +3922,16 @@
       <c r="U23" s="10" t="s">
         <v>195</v>
       </c>
-      <c r="V23" s="108">
+      <c r="V23" s="88">
         <v>9512.0900050500404</v>
       </c>
       <c r="W23" s="48">
         <v>5904.2712504522642</v>
       </c>
-      <c r="X23" s="98">
+      <c r="X23" s="84">
         <v>1185649867.7650199</v>
       </c>
-      <c r="Y23" s="98">
+      <c r="Y23" s="84">
         <v>15141.3494668729</v>
       </c>
       <c r="Z23" s="17" t="s">
@@ -3976,7 +3955,7 @@
       <c r="D24" s="11" t="s">
         <v>94</v>
       </c>
-      <c r="E24" s="82" t="s">
+      <c r="E24" s="76" t="s">
         <v>23</v>
       </c>
       <c r="F24" s="12">
@@ -3990,16 +3969,16 @@
       </c>
       <c r="I24" s="22"/>
       <c r="J24" s="13"/>
-      <c r="K24" s="75">
+      <c r="K24" s="70">
         <v>643.21000032770746</v>
       </c>
       <c r="L24" s="46">
         <v>643.21000032770746</v>
       </c>
-      <c r="M24" s="92">
+      <c r="M24" s="81">
         <v>1168969818.60271</v>
       </c>
-      <c r="N24" s="92">
+      <c r="N24" s="81">
         <v>15326.5723219425</v>
       </c>
       <c r="O24" s="23" t="s">
@@ -4021,16 +4000,16 @@
         <v>26</v>
       </c>
       <c r="U24" s="10"/>
-      <c r="V24" s="108">
+      <c r="V24" s="88">
         <v>311.99999998675048</v>
       </c>
       <c r="W24" s="48">
         <v>677.65142841758222</v>
       </c>
-      <c r="X24" s="98">
+      <c r="X24" s="84">
         <v>1203160495.6277101</v>
       </c>
-      <c r="Y24" s="98">
+      <c r="Y24" s="84">
         <v>14323.2915692312</v>
       </c>
       <c r="Z24" s="17" t="s">
@@ -4044,84 +4023,84 @@
       </c>
     </row>
     <row r="25" spans="1:28" s="18" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="110">
+      <c r="A25" s="90">
         <v>22</v>
       </c>
-      <c r="B25" s="159" t="s">
+      <c r="B25" s="130" t="s">
         <v>37</v>
       </c>
-      <c r="C25" s="112" t="s">
+      <c r="C25" s="92" t="s">
         <v>38</v>
       </c>
-      <c r="D25" s="113" t="s">
+      <c r="D25" s="93" t="s">
         <v>97</v>
       </c>
-      <c r="E25" s="125" t="s">
-        <v>23</v>
-      </c>
-      <c r="F25" s="115">
+      <c r="E25" s="105" t="s">
+        <v>23</v>
+      </c>
+      <c r="F25" s="95">
         <v>55.12618294</v>
       </c>
-      <c r="G25" s="115">
+      <c r="G25" s="95">
         <v>44.006421072666669</v>
       </c>
-      <c r="H25" s="160" t="s">
+      <c r="H25" s="131" t="s">
         <v>25</v>
       </c>
-      <c r="I25" s="161" t="s">
+      <c r="I25" s="132" t="s">
         <v>26</v>
       </c>
-      <c r="J25" s="116"/>
-      <c r="K25" s="117">
+      <c r="J25" s="96"/>
+      <c r="K25" s="97">
         <v>48.419999988213831</v>
       </c>
-      <c r="L25" s="118">
+      <c r="L25" s="98">
         <v>53.263999983194687</v>
       </c>
-      <c r="M25" s="119">
+      <c r="M25" s="99">
         <v>1173242260.8866701</v>
       </c>
-      <c r="N25" s="119">
+      <c r="N25" s="99">
         <v>15729.4413218752</v>
       </c>
-      <c r="O25" s="120" t="s">
+      <c r="O25" s="100" t="s">
         <v>98</v>
       </c>
-      <c r="P25" s="112" t="s">
-        <v>23</v>
-      </c>
-      <c r="Q25" s="121">
+      <c r="P25" s="92" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q25" s="101">
         <v>51.509602039999997</v>
       </c>
-      <c r="R25" s="121">
+      <c r="R25" s="101">
         <v>54.179899413999998</v>
       </c>
-      <c r="S25" s="160" t="s">
+      <c r="S25" s="131" t="s">
         <v>25</v>
       </c>
-      <c r="T25" s="162" t="s">
+      <c r="T25" s="133" t="s">
         <v>99</v>
       </c>
-      <c r="U25" s="112"/>
-      <c r="V25" s="122">
+      <c r="U25" s="92"/>
+      <c r="V25" s="102">
         <v>109.00000001490235</v>
       </c>
-      <c r="W25" s="123">
+      <c r="W25" s="103">
         <v>56.955333329275163</v>
       </c>
-      <c r="X25" s="124">
+      <c r="X25" s="104">
         <v>1161894612.3958299</v>
       </c>
-      <c r="Y25" s="124">
+      <c r="Y25" s="104">
         <v>15269.1620783611</v>
       </c>
-      <c r="Z25" s="125" t="s">
+      <c r="Z25" s="105" t="s">
         <v>190</v>
       </c>
-      <c r="AA25" s="116" t="s">
+      <c r="AA25" s="96" t="s">
         <v>100</v>
       </c>
-      <c r="AB25" s="126" t="s">
+      <c r="AB25" s="106" t="s">
         <v>101</v>
       </c>
     </row>
@@ -4129,10 +4108,10 @@
       <c r="A26" s="8" t="s">
         <v>222</v>
       </c>
-      <c r="B26" s="127" t="s">
+      <c r="B26" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="C26" s="127" t="s">
+      <c r="C26" s="19" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="11" t="s">
@@ -4141,64 +4120,64 @@
       <c r="E26" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="F26" s="128">
+      <c r="F26" s="12">
         <v>56.200157140000002</v>
       </c>
-      <c r="G26" s="128">
+      <c r="G26" s="12">
         <v>64.052863704999993</v>
       </c>
-      <c r="H26" s="129" t="s">
+      <c r="H26" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="I26" s="129"/>
-      <c r="J26" s="129"/>
-      <c r="K26" s="75">
+      <c r="I26" s="13"/>
+      <c r="J26" s="13"/>
+      <c r="K26" s="70">
         <v>20.630000001275377</v>
       </c>
       <c r="L26" s="46">
         <v>40.632500003026536</v>
       </c>
-      <c r="M26" s="92">
+      <c r="M26" s="81">
         <v>1152101287.4105899</v>
       </c>
-      <c r="N26" s="92">
+      <c r="N26" s="81">
         <v>15790.941415650201</v>
       </c>
       <c r="O26" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="P26" s="130" t="s">
-        <v>23</v>
-      </c>
-      <c r="Q26" s="131">
+      <c r="P26" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q26" s="16">
         <v>70.324756780000001</v>
       </c>
-      <c r="R26" s="131">
+      <c r="R26" s="16">
         <v>67.520182812352942</v>
       </c>
-      <c r="S26" s="127" t="s">
+      <c r="S26" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="T26" s="132" t="s">
+      <c r="T26" s="107" t="s">
         <v>57</v>
       </c>
-      <c r="U26" s="130"/>
-      <c r="V26" s="108">
+      <c r="U26" s="10"/>
+      <c r="V26" s="88">
         <v>23.600000001624441</v>
       </c>
       <c r="W26" s="48">
         <v>30.66699999793893</v>
       </c>
-      <c r="X26" s="98">
+      <c r="X26" s="84">
         <v>1115395380.4872899</v>
       </c>
-      <c r="Y26" s="98">
+      <c r="Y26" s="84">
         <v>14128.886124835601</v>
       </c>
       <c r="Z26" s="17" t="s">
         <v>190</v>
       </c>
-      <c r="AA26" s="129" t="s">
+      <c r="AA26" s="13" t="s">
         <v>104</v>
       </c>
       <c r="AB26" s="14" t="s">
@@ -4209,10 +4188,10 @@
       <c r="A27" s="8">
         <v>24</v>
       </c>
-      <c r="B27" s="127" t="s">
+      <c r="B27" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="C27" s="127" t="s">
+      <c r="C27" s="19" t="s">
         <v>21</v>
       </c>
       <c r="D27" s="11" t="s">
@@ -4221,64 +4200,64 @@
       <c r="E27" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="F27" s="128">
+      <c r="F27" s="12">
         <v>58.48422832</v>
       </c>
-      <c r="G27" s="128">
+      <c r="G27" s="12">
         <v>62.436892557363635</v>
       </c>
-      <c r="H27" s="129" t="s">
+      <c r="H27" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="I27" s="129"/>
-      <c r="J27" s="129"/>
-      <c r="K27" s="75">
+      <c r="I27" s="13"/>
+      <c r="J27" s="13"/>
+      <c r="K27" s="70">
         <v>9.0999999932719593</v>
       </c>
       <c r="L27" s="46">
         <v>5.5148623860335233</v>
       </c>
-      <c r="M27" s="92">
+      <c r="M27" s="81">
         <v>1141634273.41225</v>
       </c>
-      <c r="N27" s="92">
+      <c r="N27" s="81">
         <v>14593.0250856936</v>
       </c>
       <c r="O27" s="15" t="s">
         <v>107</v>
       </c>
-      <c r="P27" s="130" t="s">
-        <v>23</v>
-      </c>
-      <c r="Q27" s="131">
+      <c r="P27" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q27" s="16">
         <v>65.621511339999998</v>
       </c>
-      <c r="R27" s="131">
+      <c r="R27" s="16">
         <v>63.537957311374974</v>
       </c>
-      <c r="S27" s="127" t="s">
+      <c r="S27" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="T27" s="134" t="s">
+      <c r="T27" s="45" t="s">
         <v>108</v>
       </c>
-      <c r="U27" s="130"/>
-      <c r="V27" s="108">
+      <c r="U27" s="10"/>
+      <c r="V27" s="88">
         <v>4.2400000039761361</v>
       </c>
       <c r="W27" s="48">
         <v>4.5303821654292395</v>
       </c>
-      <c r="X27" s="98">
+      <c r="X27" s="84">
         <v>1104594382.45701</v>
       </c>
-      <c r="Y27" s="98">
+      <c r="Y27" s="84">
         <v>14572.5869919005</v>
       </c>
       <c r="Z27" s="17" t="s">
         <v>190</v>
       </c>
-      <c r="AA27" s="129" t="s">
+      <c r="AA27" s="13" t="s">
         <v>104</v>
       </c>
       <c r="AB27" s="14" t="s">
@@ -4289,74 +4268,74 @@
       <c r="A28" s="8">
         <v>25</v>
       </c>
-      <c r="B28" s="163" t="s">
+      <c r="B28" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="C28" s="130" t="s">
+      <c r="C28" s="10" t="s">
         <v>14</v>
       </c>
       <c r="D28" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="E28" s="82" t="s">
-        <v>23</v>
-      </c>
-      <c r="F28" s="128">
+      <c r="E28" s="76" t="s">
+        <v>23</v>
+      </c>
+      <c r="F28" s="12">
         <v>41.401621730000002</v>
       </c>
-      <c r="G28" s="128">
+      <c r="G28" s="12">
         <v>32.403629820555551</v>
       </c>
-      <c r="H28" s="136" t="s">
+      <c r="H28" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="I28" s="136"/>
-      <c r="J28" s="129"/>
-      <c r="K28" s="75">
+      <c r="I28" s="22"/>
+      <c r="J28" s="13"/>
+      <c r="K28" s="70">
         <v>403.32000044845677</v>
       </c>
       <c r="L28" s="46">
         <v>454.94799984267843</v>
       </c>
-      <c r="M28" s="92">
+      <c r="M28" s="81">
         <v>1154731734.1382799</v>
       </c>
-      <c r="N28" s="92">
+      <c r="N28" s="81">
         <v>14213.6000546123</v>
       </c>
       <c r="O28" s="23" t="s">
         <v>111</v>
       </c>
-      <c r="P28" s="137" t="s">
-        <v>23</v>
-      </c>
-      <c r="Q28" s="131">
+      <c r="P28" s="24" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q28" s="16">
         <v>32.992022550000002</v>
       </c>
-      <c r="R28" s="131">
+      <c r="R28" s="16">
         <v>27.252593251384223</v>
       </c>
-      <c r="S28" s="137" t="s">
+      <c r="S28" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="T28" s="137"/>
-      <c r="U28" s="130"/>
-      <c r="V28" s="108">
+      <c r="T28" s="24"/>
+      <c r="U28" s="10"/>
+      <c r="V28" s="88">
         <v>586.37000037141206</v>
       </c>
       <c r="W28" s="48">
         <v>379.93670330746147</v>
       </c>
-      <c r="X28" s="98">
+      <c r="X28" s="84">
         <v>1245600645.9167099</v>
       </c>
-      <c r="Y28" s="98">
+      <c r="Y28" s="84">
         <v>16339.15942532</v>
       </c>
       <c r="Z28" s="17" t="s">
         <v>191</v>
       </c>
-      <c r="AA28" s="129" t="s">
+      <c r="AA28" s="13" t="s">
         <v>112</v>
       </c>
       <c r="AB28" s="14"/>
@@ -4365,78 +4344,78 @@
       <c r="A29" s="8">
         <v>26</v>
       </c>
-      <c r="B29" s="163" t="s">
+      <c r="B29" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="C29" s="130" t="s">
+      <c r="C29" s="10" t="s">
         <v>38</v>
       </c>
       <c r="D29" s="11" t="s">
         <v>113</v>
       </c>
-      <c r="E29" s="82" t="s">
-        <v>23</v>
-      </c>
-      <c r="F29" s="128">
+      <c r="E29" s="76" t="s">
+        <v>23</v>
+      </c>
+      <c r="F29" s="12">
         <v>38.016314819999998</v>
       </c>
-      <c r="G29" s="128">
+      <c r="G29" s="12">
         <v>34.53754543208052</v>
       </c>
-      <c r="H29" s="127" t="s">
+      <c r="H29" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="I29" s="164" t="s">
+      <c r="I29" s="43" t="s">
         <v>26</v>
       </c>
-      <c r="J29" s="129"/>
-      <c r="K29" s="75">
+      <c r="J29" s="13"/>
+      <c r="K29" s="70">
         <v>4729.2699984324208</v>
       </c>
       <c r="L29" s="46">
         <v>765.12317250772571</v>
       </c>
-      <c r="M29" s="92">
+      <c r="M29" s="81">
         <v>1211838455.5174</v>
       </c>
-      <c r="N29" s="92">
+      <c r="N29" s="81">
         <v>16085.0145200354</v>
       </c>
       <c r="O29" s="23" t="s">
         <v>114</v>
       </c>
-      <c r="P29" s="137" t="s">
-        <v>23</v>
-      </c>
-      <c r="Q29" s="131">
+      <c r="P29" s="24" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q29" s="16">
         <v>36.974460980000003</v>
       </c>
-      <c r="R29" s="131">
+      <c r="R29" s="16">
         <v>32.650297077837834</v>
       </c>
-      <c r="S29" s="127" t="s">
+      <c r="S29" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="T29" s="132" t="s">
+      <c r="T29" s="107" t="s">
         <v>115</v>
       </c>
-      <c r="U29" s="130"/>
-      <c r="V29" s="108">
+      <c r="U29" s="10"/>
+      <c r="V29" s="88">
         <v>4247.9699998908764</v>
       </c>
       <c r="W29" s="48">
         <v>1862.8580552863245</v>
       </c>
-      <c r="X29" s="98">
+      <c r="X29" s="84">
         <v>1177796155.25647</v>
       </c>
-      <c r="Y29" s="98">
+      <c r="Y29" s="84">
         <v>15299.136525067001</v>
       </c>
       <c r="Z29" s="17" t="s">
         <v>191</v>
       </c>
-      <c r="AA29" s="129" t="s">
+      <c r="AA29" s="13" t="s">
         <v>116</v>
       </c>
       <c r="AB29" s="14" t="s">
@@ -4447,74 +4426,74 @@
       <c r="A30" s="8">
         <v>27</v>
       </c>
-      <c r="B30" s="163" t="s">
+      <c r="B30" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="C30" s="130" t="s">
+      <c r="C30" s="10" t="s">
         <v>14</v>
       </c>
       <c r="D30" s="21" t="s">
         <v>118</v>
       </c>
-      <c r="E30" s="82" t="s">
+      <c r="E30" s="76" t="s">
         <v>119</v>
       </c>
-      <c r="F30" s="128">
+      <c r="F30" s="12">
         <v>25.329944510000001</v>
       </c>
-      <c r="G30" s="128">
+      <c r="G30" s="12">
         <v>27.327156512500004</v>
       </c>
-      <c r="H30" s="136" t="s">
+      <c r="H30" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="I30" s="136"/>
-      <c r="J30" s="129"/>
-      <c r="K30" s="75">
+      <c r="I30" s="22"/>
+      <c r="J30" s="13"/>
+      <c r="K30" s="70">
         <v>51.099999984149434</v>
       </c>
       <c r="L30" s="46">
         <v>46.222499984848938</v>
       </c>
-      <c r="M30" s="92">
+      <c r="M30" s="81">
         <v>1102982884.63237</v>
       </c>
-      <c r="N30" s="92">
+      <c r="N30" s="81">
         <v>14693.462212467401</v>
       </c>
       <c r="O30" s="23" t="s">
         <v>120</v>
       </c>
-      <c r="P30" s="137" t="s">
+      <c r="P30" s="24" t="s">
         <v>119</v>
       </c>
-      <c r="Q30" s="131">
+      <c r="Q30" s="16">
         <v>32.046508209999999</v>
       </c>
-      <c r="R30" s="131">
+      <c r="R30" s="16">
         <v>30.799338644999999</v>
       </c>
-      <c r="S30" s="137" t="s">
+      <c r="S30" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="T30" s="137"/>
-      <c r="U30" s="130"/>
-      <c r="V30" s="108">
+      <c r="T30" s="24"/>
+      <c r="U30" s="10"/>
+      <c r="V30" s="88">
         <v>52.699999974208303</v>
       </c>
       <c r="W30" s="48">
         <v>49.100000005065922</v>
       </c>
-      <c r="X30" s="98">
+      <c r="X30" s="84">
         <v>1121977045.1545</v>
       </c>
-      <c r="Y30" s="98">
+      <c r="Y30" s="84">
         <v>16270.382051933801</v>
       </c>
       <c r="Z30" s="17" t="s">
         <v>192</v>
       </c>
-      <c r="AA30" s="129" t="s">
+      <c r="AA30" s="13" t="s">
         <v>121</v>
       </c>
       <c r="AB30" s="14" t="s">
@@ -4522,233 +4501,233 @@
       </c>
     </row>
     <row r="31" spans="1:28" s="18" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="138">
+      <c r="A31" s="109">
         <v>28</v>
       </c>
-      <c r="B31" s="139" t="s">
+      <c r="B31" s="110" t="s">
         <v>37</v>
       </c>
-      <c r="C31" s="140" t="s">
+      <c r="C31" s="111" t="s">
         <v>14</v>
       </c>
-      <c r="D31" s="165" t="s">
+      <c r="D31" s="134" t="s">
         <v>123</v>
       </c>
-      <c r="E31" s="142" t="s">
-        <v>23</v>
-      </c>
-      <c r="F31" s="143">
+      <c r="E31" s="113" t="s">
+        <v>23</v>
+      </c>
+      <c r="F31" s="114">
         <v>38.812413169999999</v>
       </c>
-      <c r="G31" s="143">
+      <c r="G31" s="114">
         <v>38.003943886666669</v>
       </c>
-      <c r="H31" s="166" t="s">
+      <c r="H31" s="135" t="s">
         <v>16</v>
       </c>
-      <c r="I31" s="166"/>
-      <c r="J31" s="146"/>
-      <c r="K31" s="147">
+      <c r="I31" s="135"/>
+      <c r="J31" s="117"/>
+      <c r="K31" s="118">
         <v>54.999999937407871</v>
       </c>
-      <c r="L31" s="148">
+      <c r="L31" s="119">
         <v>60.236666619969021</v>
       </c>
-      <c r="M31" s="149">
+      <c r="M31" s="120">
         <v>1101198106.05212</v>
       </c>
-      <c r="N31" s="149">
+      <c r="N31" s="120">
         <v>14522.656300122</v>
       </c>
-      <c r="O31" s="167" t="s">
+      <c r="O31" s="136" t="s">
         <v>124</v>
       </c>
-      <c r="P31" s="151" t="s">
-        <v>23</v>
-      </c>
-      <c r="Q31" s="152">
+      <c r="P31" s="122" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q31" s="123">
         <v>34.455690359999998</v>
       </c>
-      <c r="R31" s="152">
+      <c r="R31" s="123">
         <v>37.089448389250002</v>
       </c>
-      <c r="S31" s="151" t="s">
+      <c r="S31" s="122" t="s">
         <v>16</v>
       </c>
-      <c r="T31" s="151"/>
-      <c r="U31" s="140"/>
-      <c r="V31" s="154">
+      <c r="T31" s="122"/>
+      <c r="U31" s="111"/>
+      <c r="V31" s="125">
         <v>113.9999999116778</v>
       </c>
-      <c r="W31" s="155">
+      <c r="W31" s="126">
         <v>92.844249987846567</v>
       </c>
-      <c r="X31" s="156">
+      <c r="X31" s="127">
         <v>1109183747.2513199</v>
       </c>
-      <c r="Y31" s="156">
+      <c r="Y31" s="127">
         <v>15791.063124848</v>
       </c>
-      <c r="Z31" s="157" t="s">
+      <c r="Z31" s="128" t="s">
         <v>192</v>
       </c>
-      <c r="AA31" s="146" t="s">
+      <c r="AA31" s="117" t="s">
         <v>125</v>
       </c>
-      <c r="AB31" s="158" t="s">
+      <c r="AB31" s="129" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="32" spans="1:28" s="18" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="110">
+      <c r="A32" s="90">
         <v>29</v>
       </c>
-      <c r="B32" s="159" t="s">
+      <c r="B32" s="130" t="s">
         <v>37</v>
       </c>
-      <c r="C32" s="112" t="s">
+      <c r="C32" s="92" t="s">
         <v>14</v>
       </c>
-      <c r="D32" s="168" t="s">
+      <c r="D32" s="137" t="s">
         <v>127</v>
       </c>
-      <c r="E32" s="169" t="s">
-        <v>23</v>
-      </c>
-      <c r="F32" s="115">
+      <c r="E32" s="138" t="s">
+        <v>23</v>
+      </c>
+      <c r="F32" s="95">
         <v>21.665198849999999</v>
       </c>
-      <c r="G32" s="115">
+      <c r="G32" s="95">
         <v>18.314243875254231</v>
       </c>
-      <c r="H32" s="170" t="s">
+      <c r="H32" s="139" t="s">
         <v>16</v>
       </c>
-      <c r="I32" s="170"/>
-      <c r="J32" s="170"/>
-      <c r="K32" s="117">
+      <c r="I32" s="139"/>
+      <c r="J32" s="139"/>
+      <c r="K32" s="97">
         <v>2371.5799989204465</v>
       </c>
-      <c r="L32" s="118">
+      <c r="L32" s="98">
         <v>926.92799996813983</v>
       </c>
-      <c r="M32" s="119">
+      <c r="M32" s="99">
         <v>1121184390.2305801</v>
       </c>
-      <c r="N32" s="119">
+      <c r="N32" s="99">
         <v>14639.391298677499</v>
       </c>
-      <c r="O32" s="171" t="s">
+      <c r="O32" s="140" t="s">
         <v>128</v>
       </c>
-      <c r="P32" s="172" t="s">
-        <v>23</v>
-      </c>
-      <c r="Q32" s="121">
+      <c r="P32" s="141" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q32" s="101">
         <v>20.54886947</v>
       </c>
-      <c r="R32" s="121">
+      <c r="R32" s="101">
         <v>20.641531104999999</v>
       </c>
-      <c r="S32" s="172" t="s">
+      <c r="S32" s="141" t="s">
         <v>16</v>
       </c>
-      <c r="T32" s="172"/>
-      <c r="U32" s="112"/>
-      <c r="V32" s="122">
+      <c r="T32" s="141"/>
+      <c r="U32" s="92"/>
+      <c r="V32" s="102">
         <v>3999.9999969793548</v>
       </c>
-      <c r="W32" s="123">
+      <c r="W32" s="103">
         <v>3871.8099993730311</v>
       </c>
-      <c r="X32" s="124">
+      <c r="X32" s="104">
         <v>1102479368.81042</v>
       </c>
-      <c r="Y32" s="124">
+      <c r="Y32" s="104">
         <v>15890.143749085601</v>
       </c>
-      <c r="Z32" s="125" t="s">
+      <c r="Z32" s="105" t="s">
         <v>192</v>
       </c>
-      <c r="AA32" s="116" t="s">
+      <c r="AA32" s="96" t="s">
         <v>129</v>
       </c>
-      <c r="AB32" s="126"/>
+      <c r="AB32" s="106"/>
     </row>
     <row r="33" spans="1:33" s="18" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A33" s="8">
         <v>30</v>
       </c>
-      <c r="B33" s="127" t="s">
+      <c r="B33" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="C33" s="127" t="s">
+      <c r="C33" s="19" t="s">
         <v>21</v>
       </c>
       <c r="D33" s="11" t="s">
         <v>130</v>
       </c>
-      <c r="E33" s="82" t="s">
-        <v>23</v>
-      </c>
-      <c r="F33" s="128">
+      <c r="E33" s="76" t="s">
+        <v>23</v>
+      </c>
+      <c r="F33" s="12">
         <v>42.409350869999997</v>
       </c>
-      <c r="G33" s="128">
+      <c r="G33" s="12">
         <v>28.933694254705888</v>
       </c>
-      <c r="H33" s="136" t="s">
+      <c r="H33" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="I33" s="136"/>
-      <c r="J33" s="136"/>
-      <c r="K33" s="75">
+      <c r="I33" s="22"/>
+      <c r="J33" s="22"/>
+      <c r="K33" s="70">
         <v>96.290000065230885</v>
       </c>
       <c r="L33" s="46">
         <v>134.00352939393434</v>
       </c>
-      <c r="M33" s="92">
+      <c r="M33" s="81">
         <v>1146510011.74174</v>
       </c>
-      <c r="N33" s="92">
+      <c r="N33" s="81">
         <v>16099.8940049423</v>
       </c>
       <c r="O33" s="15" t="s">
         <v>131</v>
       </c>
-      <c r="P33" s="137" t="s">
-        <v>23</v>
-      </c>
-      <c r="Q33" s="131">
+      <c r="P33" s="24" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q33" s="16">
         <v>40.104351430000001</v>
       </c>
-      <c r="R33" s="131">
+      <c r="R33" s="16">
         <v>33.095598666923074</v>
       </c>
-      <c r="S33" s="127" t="s">
+      <c r="S33" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="T33" s="134" t="s">
+      <c r="T33" s="45" t="s">
         <v>60</v>
       </c>
-      <c r="U33" s="137"/>
-      <c r="V33" s="108">
+      <c r="U33" s="24"/>
+      <c r="V33" s="88">
         <v>42.400000039761373</v>
       </c>
       <c r="W33" s="48">
         <v>35.657307697429765</v>
       </c>
-      <c r="X33" s="98">
+      <c r="X33" s="84">
         <v>1082966621.8972299</v>
       </c>
-      <c r="Y33" s="98">
+      <c r="Y33" s="84">
         <v>14449.2059778231</v>
       </c>
       <c r="Z33" s="17" t="s">
         <v>192</v>
       </c>
-      <c r="AA33" s="129" t="s">
+      <c r="AA33" s="13" t="s">
         <v>132</v>
       </c>
       <c r="AB33" s="14"/>
@@ -4757,74 +4736,74 @@
       <c r="A34" s="8">
         <v>31</v>
       </c>
-      <c r="B34" s="163" t="s">
+      <c r="B34" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="C34" s="130" t="s">
+      <c r="C34" s="10" t="s">
         <v>14</v>
       </c>
       <c r="D34" s="11" t="s">
         <v>182</v>
       </c>
-      <c r="E34" s="82" t="s">
-        <v>23</v>
-      </c>
-      <c r="F34" s="128">
+      <c r="E34" s="76" t="s">
+        <v>23</v>
+      </c>
+      <c r="F34" s="12">
         <v>16.289022079999999</v>
       </c>
-      <c r="G34" s="128">
+      <c r="G34" s="12">
         <v>21.259630229457397</v>
       </c>
-      <c r="H34" s="136" t="s">
+      <c r="H34" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="I34" s="136"/>
-      <c r="J34" s="136"/>
-      <c r="K34" s="75">
+      <c r="I34" s="22"/>
+      <c r="J34" s="22"/>
+      <c r="K34" s="70">
         <v>25.549999972306377</v>
       </c>
       <c r="L34" s="46">
         <v>81.135565598717392</v>
       </c>
-      <c r="M34" s="92">
+      <c r="M34" s="81">
         <v>1168452230.3999701</v>
       </c>
-      <c r="N34" s="92">
+      <c r="N34" s="81">
         <v>14405.0486215031</v>
       </c>
       <c r="O34" s="23" t="s">
         <v>133</v>
       </c>
-      <c r="P34" s="137" t="s">
-        <v>23</v>
-      </c>
-      <c r="Q34" s="131">
+      <c r="P34" s="24" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q34" s="16">
         <v>19.638930760000001</v>
       </c>
-      <c r="R34" s="131">
+      <c r="R34" s="16">
         <v>22.459104802352943</v>
       </c>
-      <c r="S34" s="137" t="s">
+      <c r="S34" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="T34" s="137"/>
-      <c r="U34" s="137"/>
-      <c r="V34" s="108">
+      <c r="T34" s="24"/>
+      <c r="U34" s="24"/>
+      <c r="V34" s="88">
         <v>46.799999992012332</v>
       </c>
       <c r="W34" s="48">
         <v>27.407058824246327</v>
       </c>
-      <c r="X34" s="98">
+      <c r="X34" s="84">
         <v>1139499084.3313301</v>
       </c>
-      <c r="Y34" s="98">
+      <c r="Y34" s="84">
         <v>15828.700782477599</v>
       </c>
       <c r="Z34" s="17" t="s">
         <v>192</v>
       </c>
-      <c r="AA34" s="129" t="s">
+      <c r="AA34" s="13" t="s">
         <v>134</v>
       </c>
       <c r="AB34" s="14"/>
@@ -4833,74 +4812,74 @@
       <c r="A35" s="8">
         <v>32</v>
       </c>
-      <c r="B35" s="163" t="s">
+      <c r="B35" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="C35" s="130" t="s">
+      <c r="C35" s="10" t="s">
         <v>14</v>
       </c>
       <c r="D35" s="11" t="s">
         <v>135</v>
       </c>
-      <c r="E35" s="82" t="s">
-        <v>23</v>
-      </c>
-      <c r="F35" s="128">
+      <c r="E35" s="76" t="s">
+        <v>23</v>
+      </c>
+      <c r="F35" s="12">
         <v>10.6789811</v>
       </c>
-      <c r="G35" s="128">
+      <c r="G35" s="12">
         <v>10.6789811</v>
       </c>
-      <c r="H35" s="136" t="s">
+      <c r="H35" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="I35" s="136"/>
-      <c r="J35" s="136"/>
-      <c r="K35" s="75">
+      <c r="I35" s="22"/>
+      <c r="J35" s="22"/>
+      <c r="K35" s="70">
         <v>1400.0000010372382</v>
       </c>
       <c r="L35" s="46">
         <v>1400.0000010372382</v>
       </c>
-      <c r="M35" s="92">
+      <c r="M35" s="81">
         <v>1161341873.44103</v>
       </c>
-      <c r="N35" s="92">
+      <c r="N35" s="81">
         <v>15133.446081604699</v>
       </c>
       <c r="O35" s="23" t="s">
         <v>136</v>
       </c>
-      <c r="P35" s="137" t="s">
-        <v>23</v>
-      </c>
-      <c r="Q35" s="131">
+      <c r="P35" s="24" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q35" s="16">
         <v>10.686582570000001</v>
       </c>
-      <c r="R35" s="131">
+      <c r="R35" s="16">
         <v>10.686582570000001</v>
       </c>
-      <c r="S35" s="137" t="s">
+      <c r="S35" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="T35" s="137"/>
-      <c r="U35" s="137"/>
-      <c r="V35" s="108">
+      <c r="T35" s="24"/>
+      <c r="U35" s="24"/>
+      <c r="V35" s="88">
         <v>1297.9999986121711</v>
       </c>
       <c r="W35" s="48">
         <v>1297.9999986121711</v>
       </c>
-      <c r="X35" s="98">
+      <c r="X35" s="84">
         <v>1164886917.7786801</v>
       </c>
-      <c r="Y35" s="98">
+      <c r="Y35" s="84">
         <v>15841.9070414419</v>
       </c>
       <c r="Z35" s="17" t="s">
         <v>193</v>
       </c>
-      <c r="AA35" s="129" t="s">
+      <c r="AA35" s="13" t="s">
         <v>137</v>
       </c>
       <c r="AB35" s="14" t="s">
@@ -4911,76 +4890,76 @@
       <c r="A36" s="8" t="s">
         <v>223</v>
       </c>
-      <c r="B36" s="127" t="s">
+      <c r="B36" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="C36" s="127" t="s">
+      <c r="C36" s="19" t="s">
         <v>21</v>
       </c>
       <c r="D36" s="21" t="s">
         <v>139</v>
       </c>
-      <c r="E36" s="82" t="s">
-        <v>23</v>
-      </c>
-      <c r="F36" s="128">
+      <c r="E36" s="76" t="s">
+        <v>23</v>
+      </c>
+      <c r="F36" s="12">
         <v>18.919017530000001</v>
       </c>
-      <c r="G36" s="128">
+      <c r="G36" s="12">
         <v>19.119666978749997</v>
       </c>
-      <c r="H36" s="136" t="s">
+      <c r="H36" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="I36" s="136"/>
-      <c r="J36" s="136"/>
-      <c r="K36" s="75">
+      <c r="I36" s="22"/>
+      <c r="J36" s="22"/>
+      <c r="K36" s="70">
         <v>623.58000047396831</v>
       </c>
       <c r="L36" s="46">
         <v>379.97500017522975</v>
       </c>
-      <c r="M36" s="92">
+      <c r="M36" s="81">
         <v>1169964629.2257299</v>
       </c>
-      <c r="N36" s="92">
+      <c r="N36" s="81">
         <v>15649.2477742551</v>
       </c>
       <c r="O36" s="23" t="s">
         <v>140</v>
       </c>
-      <c r="P36" s="137" t="s">
-        <v>23</v>
-      </c>
-      <c r="Q36" s="131">
+      <c r="P36" s="24" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q36" s="16">
         <v>55.422399259999999</v>
       </c>
-      <c r="R36" s="131">
+      <c r="R36" s="16">
         <v>46.4742153322807</v>
       </c>
-      <c r="S36" s="127" t="s">
+      <c r="S36" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="T36" s="132" t="s">
+      <c r="T36" s="107" t="s">
         <v>115</v>
       </c>
-      <c r="U36" s="137"/>
-      <c r="V36" s="108">
+      <c r="U36" s="24"/>
+      <c r="V36" s="88">
         <v>759.94999941293793</v>
       </c>
       <c r="W36" s="48">
         <v>393.82160713452311</v>
       </c>
-      <c r="X36" s="98">
+      <c r="X36" s="84">
         <v>1164244529.0397999</v>
       </c>
-      <c r="Y36" s="98">
+      <c r="Y36" s="84">
         <v>15111.1199700211</v>
       </c>
       <c r="Z36" s="17" t="s">
         <v>193</v>
       </c>
-      <c r="AA36" s="129" t="s">
+      <c r="AA36" s="13" t="s">
         <v>141</v>
       </c>
       <c r="AB36" s="14" t="s">
@@ -4991,155 +4970,155 @@
       <c r="A37" s="8">
         <v>34</v>
       </c>
-      <c r="B37" s="127" t="s">
+      <c r="B37" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="C37" s="127" t="s">
+      <c r="C37" s="19" t="s">
         <v>21</v>
       </c>
       <c r="D37" s="21" t="s">
         <v>143</v>
       </c>
-      <c r="E37" s="82" t="s">
-        <v>23</v>
-      </c>
-      <c r="F37" s="128">
+      <c r="E37" s="76" t="s">
+        <v>23</v>
+      </c>
+      <c r="F37" s="12">
         <v>34.48747281</v>
       </c>
-      <c r="G37" s="128">
+      <c r="G37" s="12">
         <v>29.941332736666666</v>
       </c>
-      <c r="H37" s="136" t="s">
+      <c r="H37" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="I37" s="136"/>
-      <c r="J37" s="136"/>
-      <c r="K37" s="75">
+      <c r="I37" s="22"/>
+      <c r="J37" s="22"/>
+      <c r="K37" s="70">
         <v>862.96999938452666</v>
       </c>
       <c r="L37" s="46">
         <v>1007.6766666469121</v>
       </c>
-      <c r="M37" s="92">
+      <c r="M37" s="81">
         <v>1076982615.9507599</v>
       </c>
-      <c r="N37" s="92">
+      <c r="N37" s="81">
         <v>15176.527237910501</v>
       </c>
       <c r="O37" s="23" t="s">
         <v>144</v>
       </c>
-      <c r="P37" s="137" t="s">
-        <v>23</v>
-      </c>
-      <c r="Q37" s="131">
+      <c r="P37" s="24" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q37" s="16">
         <v>50.820552210000002</v>
       </c>
-      <c r="R37" s="131">
+      <c r="R37" s="16">
         <v>40.531540337100289</v>
       </c>
-      <c r="S37" s="127" t="s">
+      <c r="S37" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="T37" s="134" t="s">
+      <c r="T37" s="45" t="s">
         <v>145</v>
       </c>
-      <c r="U37" s="137"/>
-      <c r="V37" s="108">
+      <c r="U37" s="24"/>
+      <c r="V37" s="88">
         <v>28.989999976303245</v>
       </c>
       <c r="W37" s="48">
         <v>1007.6766666469121</v>
       </c>
-      <c r="X37" s="98">
+      <c r="X37" s="84">
         <v>1101580076.9507201</v>
       </c>
-      <c r="Y37" s="98">
+      <c r="Y37" s="84">
         <v>13769.309358181799</v>
       </c>
       <c r="Z37" s="17" t="s">
         <v>193</v>
       </c>
-      <c r="AA37" s="129" t="s">
+      <c r="AA37" s="13" t="s">
         <v>146</v>
       </c>
       <c r="AB37" s="14"/>
     </row>
     <row r="38" spans="1:33" s="18" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="138">
+      <c r="A38" s="109">
         <v>35</v>
       </c>
-      <c r="B38" s="139" t="s">
+      <c r="B38" s="110" t="s">
         <v>37</v>
       </c>
-      <c r="C38" s="140" t="s">
+      <c r="C38" s="111" t="s">
         <v>14</v>
       </c>
-      <c r="D38" s="165" t="s">
+      <c r="D38" s="134" t="s">
         <v>147</v>
       </c>
-      <c r="E38" s="142" t="s">
-        <v>23</v>
-      </c>
-      <c r="F38" s="143">
+      <c r="E38" s="113" t="s">
+        <v>23</v>
+      </c>
+      <c r="F38" s="114">
         <v>15.69798372</v>
       </c>
-      <c r="G38" s="143">
+      <c r="G38" s="114">
         <v>18.463281178235292</v>
       </c>
-      <c r="H38" s="166" t="s">
+      <c r="H38" s="135" t="s">
         <v>16</v>
       </c>
-      <c r="I38" s="166"/>
-      <c r="J38" s="166"/>
-      <c r="K38" s="147">
+      <c r="I38" s="135"/>
+      <c r="J38" s="135"/>
+      <c r="K38" s="118">
         <v>16.699999994324962</v>
       </c>
-      <c r="L38" s="148">
+      <c r="L38" s="119">
         <v>15.155624995660526</v>
       </c>
-      <c r="M38" s="149">
+      <c r="M38" s="120">
         <v>1194692095.1575201</v>
       </c>
-      <c r="N38" s="149">
+      <c r="N38" s="120">
         <v>15141.628628314</v>
       </c>
-      <c r="O38" s="167" t="s">
+      <c r="O38" s="136" t="s">
         <v>148</v>
       </c>
-      <c r="P38" s="151" t="s">
-        <v>23</v>
-      </c>
-      <c r="Q38" s="152">
+      <c r="P38" s="122" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q38" s="123">
         <v>18.391934790000001</v>
       </c>
-      <c r="R38" s="152">
+      <c r="R38" s="123">
         <v>19.288713850000001</v>
       </c>
-      <c r="S38" s="151" t="s">
+      <c r="S38" s="122" t="s">
         <v>16</v>
       </c>
-      <c r="T38" s="151"/>
-      <c r="U38" s="151"/>
-      <c r="V38" s="154">
+      <c r="T38" s="122"/>
+      <c r="U38" s="122"/>
+      <c r="V38" s="125">
         <v>8.3400000069567088</v>
       </c>
-      <c r="W38" s="155">
+      <c r="W38" s="126">
         <v>9.2211111093385014</v>
       </c>
-      <c r="X38" s="156">
+      <c r="X38" s="127">
         <v>1068315062.53522</v>
       </c>
-      <c r="Y38" s="156">
+      <c r="Y38" s="127">
         <v>15067.1071498284</v>
       </c>
-      <c r="Z38" s="157" t="s">
+      <c r="Z38" s="128" t="s">
         <v>193</v>
       </c>
-      <c r="AA38" s="146" t="s">
+      <c r="AA38" s="117" t="s">
         <v>149</v>
       </c>
-      <c r="AB38" s="158" t="s">
+      <c r="AB38" s="129" t="s">
         <v>150</v>
       </c>
     </row>
@@ -5156,7 +5135,7 @@
       <c r="D39" s="21" t="s">
         <v>151</v>
       </c>
-      <c r="E39" s="81" t="s">
+      <c r="E39" s="75" t="s">
         <v>176</v>
       </c>
       <c r="F39" s="12">
@@ -5170,16 +5149,16 @@
       </c>
       <c r="I39" s="22"/>
       <c r="J39" s="22"/>
-      <c r="K39" s="75">
+      <c r="K39" s="70">
         <v>17.799999987339671</v>
       </c>
       <c r="L39" s="46">
         <v>31.105471695972899</v>
       </c>
-      <c r="M39" s="92">
+      <c r="M39" s="81">
         <v>1066557705.37684</v>
       </c>
-      <c r="N39" s="92">
+      <c r="N39" s="81">
         <v>15710.9008867053</v>
       </c>
       <c r="O39" s="23" t="s">
@@ -5199,16 +5178,16 @@
       </c>
       <c r="T39" s="24"/>
       <c r="U39" s="24"/>
-      <c r="V39" s="108">
+      <c r="V39" s="88">
         <v>33.4999999971579</v>
       </c>
       <c r="W39" s="48">
         <v>32.875682539747501</v>
       </c>
-      <c r="X39" s="98">
+      <c r="X39" s="84">
         <v>1052497871.4555</v>
       </c>
-      <c r="Y39" s="98">
+      <c r="Y39" s="84">
         <v>15850.936467269201</v>
       </c>
       <c r="Z39" s="17" t="s">
@@ -5232,7 +5211,7 @@
       <c r="D40" s="11" t="s">
         <v>154</v>
       </c>
-      <c r="E40" s="81" t="s">
+      <c r="E40" s="75" t="s">
         <v>176</v>
       </c>
       <c r="F40" s="12">
@@ -5246,16 +5225,16 @@
       </c>
       <c r="I40" s="13"/>
       <c r="J40" s="13"/>
-      <c r="K40" s="75">
+      <c r="K40" s="70">
         <v>42.150000003808309</v>
       </c>
       <c r="L40" s="46">
         <v>33.075000009872774</v>
       </c>
-      <c r="M40" s="92">
+      <c r="M40" s="81">
         <v>1064545541.59391</v>
       </c>
-      <c r="N40" s="92">
+      <c r="N40" s="81">
         <v>16939.7574130502</v>
       </c>
       <c r="O40" s="15" t="s">
@@ -5275,16 +5254,16 @@
       </c>
       <c r="T40" s="24"/>
       <c r="U40" s="10"/>
-      <c r="V40" s="108">
+      <c r="V40" s="88">
         <v>972.62000060897537</v>
       </c>
       <c r="W40" s="48">
         <v>950.31000007065586</v>
       </c>
-      <c r="X40" s="98">
+      <c r="X40" s="84">
         <v>1053652877.6775</v>
       </c>
-      <c r="Y40" s="98">
+      <c r="Y40" s="84">
         <v>15812.877962091499</v>
       </c>
       <c r="Z40" s="17" t="s">
@@ -5308,7 +5287,7 @@
       <c r="D41" s="21" t="s">
         <v>157</v>
       </c>
-      <c r="E41" s="80" t="s">
+      <c r="E41" s="74" t="s">
         <v>18</v>
       </c>
       <c r="F41" s="12">
@@ -5322,16 +5301,16 @@
       </c>
       <c r="I41" s="22"/>
       <c r="J41" s="22"/>
-      <c r="K41" s="75">
+      <c r="K41" s="70">
         <v>149.90999994399482</v>
       </c>
       <c r="L41" s="46">
         <v>88.676666603822866</v>
       </c>
-      <c r="M41" s="92">
+      <c r="M41" s="81">
         <v>1033933681.63682</v>
       </c>
-      <c r="N41" s="92">
+      <c r="N41" s="81">
         <v>15831.36356482</v>
       </c>
       <c r="O41" s="23" t="s">
@@ -5351,16 +5330,16 @@
       </c>
       <c r="T41" s="24"/>
       <c r="U41" s="24"/>
-      <c r="V41" s="108">
+      <c r="V41" s="88">
         <v>57.799999944032052</v>
       </c>
       <c r="W41" s="48">
         <v>54.030000006059637</v>
       </c>
-      <c r="X41" s="98">
+      <c r="X41" s="84">
         <v>1050341548.12155</v>
       </c>
-      <c r="Y41" s="98">
+      <c r="Y41" s="84">
         <v>16018.328104341501</v>
       </c>
       <c r="Z41" s="17" t="s">
@@ -5384,7 +5363,7 @@
       <c r="D42" s="21" t="s">
         <v>160</v>
       </c>
-      <c r="E42" s="82" t="s">
+      <c r="E42" s="76" t="s">
         <v>23</v>
       </c>
       <c r="F42" s="12">
@@ -5398,16 +5377,16 @@
       </c>
       <c r="I42" s="22"/>
       <c r="J42" s="22"/>
-      <c r="K42" s="75">
+      <c r="K42" s="70">
         <v>77.120000018685502</v>
       </c>
       <c r="L42" s="46">
         <v>141.74810809983273</v>
       </c>
-      <c r="M42" s="92">
+      <c r="M42" s="81">
         <v>1047053180.25054</v>
       </c>
-      <c r="N42" s="92">
+      <c r="N42" s="81">
         <v>15338.030147372199</v>
       </c>
       <c r="O42" s="23" t="s">
@@ -5429,16 +5408,16 @@
         <v>26</v>
       </c>
       <c r="U42" s="24"/>
-      <c r="V42" s="108">
+      <c r="V42" s="88">
         <v>448.75999963833306</v>
       </c>
       <c r="W42" s="48">
         <v>396.21203383492463</v>
       </c>
-      <c r="X42" s="98">
+      <c r="X42" s="84">
         <v>1081915449.9195199</v>
       </c>
-      <c r="Y42" s="98">
+      <c r="Y42" s="84">
         <v>14548.453900246899</v>
       </c>
       <c r="Z42" s="17" t="s">
@@ -5464,7 +5443,7 @@
       <c r="D43" s="11" t="s">
         <v>164</v>
       </c>
-      <c r="E43" s="82" t="s">
+      <c r="E43" s="76" t="s">
         <v>23</v>
       </c>
       <c r="F43" s="12">
@@ -5480,16 +5459,16 @@
         <v>165</v>
       </c>
       <c r="J43" s="22"/>
-      <c r="K43" s="75">
+      <c r="K43" s="70">
         <v>13.819999998785063</v>
       </c>
       <c r="L43" s="46">
         <v>13.819999998785063</v>
       </c>
-      <c r="M43" s="92">
+      <c r="M43" s="81">
         <v>929869190.87817395</v>
       </c>
-      <c r="N43" s="92">
+      <c r="N43" s="81">
         <v>15562.791177790899</v>
       </c>
       <c r="O43" s="23" t="s">
@@ -5511,16 +5490,16 @@
         <v>60</v>
       </c>
       <c r="U43" s="24"/>
-      <c r="V43" s="108">
+      <c r="V43" s="88">
         <v>22.199999976964538</v>
       </c>
       <c r="W43" s="48">
         <v>29.841648349399971</v>
       </c>
-      <c r="X43" s="98">
+      <c r="X43" s="84">
         <v>1087868626.26759</v>
       </c>
-      <c r="Y43" s="98">
+      <c r="Y43" s="84">
         <v>16512.6410559785</v>
       </c>
       <c r="Z43" s="17" t="s">
@@ -5544,7 +5523,7 @@
       <c r="D44" s="21" t="s">
         <v>168</v>
       </c>
-      <c r="E44" s="82" t="s">
+      <c r="E44" s="76" t="s">
         <v>23</v>
       </c>
       <c r="F44" s="12">
@@ -5558,16 +5537,16 @@
       </c>
       <c r="I44" s="22"/>
       <c r="J44" s="22"/>
-      <c r="K44" s="75">
+      <c r="K44" s="70">
         <v>12.299999987555465</v>
       </c>
       <c r="L44" s="46">
         <v>12.785853658147893</v>
       </c>
-      <c r="M44" s="92">
+      <c r="M44" s="81">
         <v>1052010832.86068</v>
       </c>
-      <c r="N44" s="92">
+      <c r="N44" s="81">
         <v>16241.278836186801</v>
       </c>
       <c r="O44" s="23" t="s">
@@ -5589,16 +5568,16 @@
         <v>145</v>
       </c>
       <c r="U44" s="24"/>
-      <c r="V44" s="108">
+      <c r="V44" s="88">
         <v>12.040000002167792</v>
       </c>
       <c r="W44" s="48">
         <v>13.000714284583239</v>
       </c>
-      <c r="X44" s="98">
+      <c r="X44" s="84">
         <v>1205791180.5840499</v>
       </c>
-      <c r="Y44" s="98">
+      <c r="Y44" s="84">
         <v>17280.731792041399</v>
       </c>
       <c r="Z44" s="17" t="s">
@@ -5624,7 +5603,7 @@
       <c r="D45" s="28" t="s">
         <v>172</v>
       </c>
-      <c r="E45" s="83" t="s">
+      <c r="E45" s="77" t="s">
         <v>23</v>
       </c>
       <c r="F45" s="30">
@@ -5638,16 +5617,16 @@
       </c>
       <c r="I45" s="29"/>
       <c r="J45" s="29"/>
-      <c r="K45" s="77">
+      <c r="K45" s="72">
         <v>24.000000015937239</v>
       </c>
       <c r="L45" s="50">
         <v>14.582835818987101</v>
       </c>
-      <c r="M45" s="95">
+      <c r="M45" s="83">
         <v>1060948464.72207</v>
       </c>
-      <c r="N45" s="95">
+      <c r="N45" s="83">
         <v>14639.061396097601</v>
       </c>
       <c r="O45" s="31" t="s">
@@ -5667,16 +5646,16 @@
       </c>
       <c r="T45" s="32"/>
       <c r="U45" s="32"/>
-      <c r="V45" s="109">
+      <c r="V45" s="89">
         <v>28.540000014547623</v>
       </c>
       <c r="W45" s="49">
         <v>19.000153846402995</v>
       </c>
-      <c r="X45" s="101">
+      <c r="X45" s="86">
         <v>1058308472.93695</v>
       </c>
-      <c r="Y45" s="101">
+      <c r="Y45" s="86">
         <v>16680.375812508199</v>
       </c>
       <c r="Z45" s="34" t="s">

</xml_diff>